<commit_message>
fix: deduplicar CAC por RUT en gráfico por región
</commit_message>
<xml_diff>
--- a/HuellaSocial_Consolidado.xlsx
+++ b/HuellaSocial_Consolidado.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Documents\Memoria\ConsolidadoTotal\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E22A03D-2636-43AF-8EA8-799228D8D29A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F316E238-B98F-4DEA-987E-2C4CAA739CCA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="3" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="360" windowWidth="23256" windowHeight="12456" firstSheet="3" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="📋 Portada" sheetId="1" r:id="rId1"/>
@@ -6834,20 +6834,11 @@
     <xf numFmtId="0" fontId="19" fillId="20" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -6868,6 +6859,16 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="13" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -6903,7 +6904,6 @@
     <xf numFmtId="0" fontId="21" fillId="20" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -7212,6 +7212,28 @@
 </a:theme>
 </file>
 
+<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
+<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
+  <wetp:taskpane dockstate="right" visibility="0" width="438" row="3">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </wetp:taskpane>
+</wetp:taskpanes>
+</file>
+
+<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{5E87ABE1-C218-4B39-9B46-C7059644922B}">
+  <we:reference id="wa200009404" version="1.0.0.8" store="es-ES" storeType="OMEX"/>
+  <we:alternateReferences>
+    <we:reference id="wa200009404" version="1.0.0.8" store="wa200009404" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties>
+    <we:property name="claude.fileId" value="&quot;f1279c13-2408-47b5-9683-9f30e728f5fb&quot;"/>
+  </we:properties>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
@@ -7247,57 +7269,57 @@
     </row>
     <row r="3" spans="1:8" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1"/>
-      <c r="B3" s="81" t="s">
-        <v>0</v>
-      </c>
-      <c r="C3" s="76"/>
-      <c r="D3" s="76"/>
-      <c r="E3" s="76"/>
-      <c r="F3" s="76"/>
-      <c r="G3" s="76"/>
-      <c r="H3" s="76"/>
+      <c r="B3" s="78" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" s="77"/>
+      <c r="D3" s="77"/>
+      <c r="E3" s="77"/>
+      <c r="F3" s="77"/>
+      <c r="G3" s="77"/>
+      <c r="H3" s="77"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="1"/>
-      <c r="B4" s="76"/>
-      <c r="C4" s="76"/>
-      <c r="D4" s="76"/>
-      <c r="E4" s="76"/>
-      <c r="F4" s="76"/>
-      <c r="G4" s="76"/>
-      <c r="H4" s="76"/>
+      <c r="B4" s="77"/>
+      <c r="C4" s="77"/>
+      <c r="D4" s="77"/>
+      <c r="E4" s="77"/>
+      <c r="F4" s="77"/>
+      <c r="G4" s="77"/>
+      <c r="H4" s="77"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="1"/>
-      <c r="B5" s="76"/>
-      <c r="C5" s="76"/>
-      <c r="D5" s="76"/>
-      <c r="E5" s="76"/>
-      <c r="F5" s="76"/>
-      <c r="G5" s="76"/>
-      <c r="H5" s="76"/>
+      <c r="B5" s="77"/>
+      <c r="C5" s="77"/>
+      <c r="D5" s="77"/>
+      <c r="E5" s="77"/>
+      <c r="F5" s="77"/>
+      <c r="G5" s="77"/>
+      <c r="H5" s="77"/>
     </row>
     <row r="6" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1"/>
-      <c r="B6" s="83" t="s">
+      <c r="B6" s="80" t="s">
         <v>1</v>
       </c>
-      <c r="C6" s="76"/>
-      <c r="D6" s="76"/>
-      <c r="E6" s="76"/>
-      <c r="F6" s="76"/>
-      <c r="G6" s="76"/>
-      <c r="H6" s="76"/>
+      <c r="C6" s="77"/>
+      <c r="D6" s="77"/>
+      <c r="E6" s="77"/>
+      <c r="F6" s="77"/>
+      <c r="G6" s="77"/>
+      <c r="H6" s="77"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="1"/>
-      <c r="B7" s="76"/>
-      <c r="C7" s="76"/>
-      <c r="D7" s="76"/>
-      <c r="E7" s="76"/>
-      <c r="F7" s="76"/>
-      <c r="G7" s="76"/>
-      <c r="H7" s="76"/>
+      <c r="B7" s="77"/>
+      <c r="C7" s="77"/>
+      <c r="D7" s="77"/>
+      <c r="E7" s="77"/>
+      <c r="F7" s="77"/>
+      <c r="G7" s="77"/>
+      <c r="H7" s="77"/>
     </row>
     <row r="8" spans="1:8" ht="6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
@@ -7321,15 +7343,15 @@
     </row>
     <row r="10" spans="1:8" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A10" s="1"/>
-      <c r="B10" s="86" t="s">
+      <c r="B10" s="83" t="s">
         <v>2</v>
       </c>
-      <c r="C10" s="76"/>
-      <c r="D10" s="76"/>
-      <c r="E10" s="76"/>
-      <c r="F10" s="76"/>
-      <c r="G10" s="76"/>
-      <c r="H10" s="76"/>
+      <c r="C10" s="77"/>
+      <c r="D10" s="77"/>
+      <c r="E10" s="77"/>
+      <c r="F10" s="77"/>
+      <c r="G10" s="77"/>
+      <c r="H10" s="77"/>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11" s="1"/>
@@ -7343,27 +7365,27 @@
     </row>
     <row r="12" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1"/>
-      <c r="B12" s="84" t="s">
+      <c r="B12" s="81" t="s">
         <v>3</v>
       </c>
-      <c r="C12" s="76"/>
-      <c r="D12" s="76"/>
-      <c r="E12" s="76"/>
-      <c r="F12" s="76"/>
-      <c r="G12" s="76"/>
-      <c r="H12" s="76"/>
+      <c r="C12" s="77"/>
+      <c r="D12" s="77"/>
+      <c r="E12" s="77"/>
+      <c r="F12" s="77"/>
+      <c r="G12" s="77"/>
+      <c r="H12" s="77"/>
     </row>
     <row r="13" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1"/>
-      <c r="B13" s="82" t="s">
+      <c r="B13" s="79" t="s">
         <v>4</v>
       </c>
-      <c r="C13" s="76"/>
-      <c r="D13" s="76"/>
-      <c r="E13" s="76"/>
-      <c r="F13" s="76"/>
-      <c r="G13" s="76"/>
-      <c r="H13" s="76"/>
+      <c r="C13" s="77"/>
+      <c r="D13" s="77"/>
+      <c r="E13" s="77"/>
+      <c r="F13" s="77"/>
+      <c r="G13" s="77"/>
+      <c r="H13" s="77"/>
     </row>
     <row r="14" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1"/>
@@ -7377,27 +7399,27 @@
     </row>
     <row r="15" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1"/>
-      <c r="B15" s="84" t="s">
+      <c r="B15" s="81" t="s">
         <v>5</v>
       </c>
-      <c r="C15" s="76"/>
-      <c r="D15" s="76"/>
-      <c r="E15" s="76"/>
-      <c r="F15" s="76"/>
-      <c r="G15" s="76"/>
-      <c r="H15" s="76"/>
+      <c r="C15" s="77"/>
+      <c r="D15" s="77"/>
+      <c r="E15" s="77"/>
+      <c r="F15" s="77"/>
+      <c r="G15" s="77"/>
+      <c r="H15" s="77"/>
     </row>
     <row r="16" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1"/>
-      <c r="B16" s="82" t="s">
+      <c r="B16" s="79" t="s">
         <v>6</v>
       </c>
-      <c r="C16" s="76"/>
-      <c r="D16" s="76"/>
-      <c r="E16" s="76"/>
-      <c r="F16" s="76"/>
-      <c r="G16" s="76"/>
-      <c r="H16" s="76"/>
+      <c r="C16" s="77"/>
+      <c r="D16" s="77"/>
+      <c r="E16" s="77"/>
+      <c r="F16" s="77"/>
+      <c r="G16" s="77"/>
+      <c r="H16" s="77"/>
     </row>
     <row r="17" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1"/>
@@ -7411,27 +7433,27 @@
     </row>
     <row r="18" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1"/>
-      <c r="B18" s="84" t="s">
+      <c r="B18" s="81" t="s">
         <v>7</v>
       </c>
-      <c r="C18" s="76"/>
-      <c r="D18" s="76"/>
-      <c r="E18" s="76"/>
-      <c r="F18" s="76"/>
-      <c r="G18" s="76"/>
-      <c r="H18" s="76"/>
+      <c r="C18" s="77"/>
+      <c r="D18" s="77"/>
+      <c r="E18" s="77"/>
+      <c r="F18" s="77"/>
+      <c r="G18" s="77"/>
+      <c r="H18" s="77"/>
     </row>
     <row r="19" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="1"/>
-      <c r="B19" s="82" t="s">
+      <c r="B19" s="79" t="s">
         <v>8</v>
       </c>
-      <c r="C19" s="76"/>
-      <c r="D19" s="76"/>
-      <c r="E19" s="76"/>
-      <c r="F19" s="76"/>
-      <c r="G19" s="76"/>
-      <c r="H19" s="76"/>
+      <c r="C19" s="77"/>
+      <c r="D19" s="77"/>
+      <c r="E19" s="77"/>
+      <c r="F19" s="77"/>
+      <c r="G19" s="77"/>
+      <c r="H19" s="77"/>
     </row>
     <row r="20" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="1"/>
@@ -7445,163 +7467,163 @@
     </row>
     <row r="21" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="1"/>
-      <c r="B21" s="84" t="s">
+      <c r="B21" s="81" t="s">
         <v>9</v>
       </c>
-      <c r="C21" s="76"/>
-      <c r="D21" s="76"/>
-      <c r="E21" s="76"/>
-      <c r="F21" s="76"/>
-      <c r="G21" s="76"/>
-      <c r="H21" s="76"/>
+      <c r="C21" s="77"/>
+      <c r="D21" s="77"/>
+      <c r="E21" s="77"/>
+      <c r="F21" s="77"/>
+      <c r="G21" s="77"/>
+      <c r="H21" s="77"/>
     </row>
     <row r="22" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="82" t="s">
+      <c r="B22" s="79" t="s">
         <v>10</v>
       </c>
-      <c r="C22" s="76"/>
-      <c r="D22" s="76"/>
-      <c r="E22" s="76"/>
-      <c r="F22" s="76"/>
-      <c r="G22" s="76"/>
-      <c r="H22" s="76"/>
+      <c r="C22" s="77"/>
+      <c r="D22" s="77"/>
+      <c r="E22" s="77"/>
+      <c r="F22" s="77"/>
+      <c r="G22" s="77"/>
+      <c r="H22" s="77"/>
     </row>
     <row r="23" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="24" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="84" t="s">
+      <c r="B24" s="81" t="s">
         <v>11</v>
       </c>
-      <c r="C24" s="76"/>
-      <c r="D24" s="76"/>
-      <c r="E24" s="76"/>
-      <c r="F24" s="76"/>
-      <c r="G24" s="76"/>
-      <c r="H24" s="76"/>
+      <c r="C24" s="77"/>
+      <c r="D24" s="77"/>
+      <c r="E24" s="77"/>
+      <c r="F24" s="77"/>
+      <c r="G24" s="77"/>
+      <c r="H24" s="77"/>
     </row>
     <row r="25" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="82" t="s">
+      <c r="B25" s="79" t="s">
         <v>12</v>
       </c>
-      <c r="C25" s="76"/>
-      <c r="D25" s="76"/>
-      <c r="E25" s="76"/>
-      <c r="F25" s="76"/>
-      <c r="G25" s="76"/>
-      <c r="H25" s="76"/>
+      <c r="C25" s="77"/>
+      <c r="D25" s="77"/>
+      <c r="E25" s="77"/>
+      <c r="F25" s="77"/>
+      <c r="G25" s="77"/>
+      <c r="H25" s="77"/>
     </row>
     <row r="26" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="27" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B27" s="84" t="s">
+      <c r="B27" s="81" t="s">
         <v>13</v>
       </c>
-      <c r="C27" s="76"/>
-      <c r="D27" s="76"/>
-      <c r="E27" s="76"/>
-      <c r="F27" s="76"/>
-      <c r="G27" s="76"/>
-      <c r="H27" s="76"/>
+      <c r="C27" s="77"/>
+      <c r="D27" s="77"/>
+      <c r="E27" s="77"/>
+      <c r="F27" s="77"/>
+      <c r="G27" s="77"/>
+      <c r="H27" s="77"/>
     </row>
     <row r="28" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B28" s="82" t="s">
+      <c r="B28" s="79" t="s">
         <v>14</v>
       </c>
-      <c r="C28" s="76"/>
-      <c r="D28" s="76"/>
-      <c r="E28" s="76"/>
-      <c r="F28" s="76"/>
-      <c r="G28" s="76"/>
-      <c r="H28" s="76"/>
+      <c r="C28" s="77"/>
+      <c r="D28" s="77"/>
+      <c r="E28" s="77"/>
+      <c r="F28" s="77"/>
+      <c r="G28" s="77"/>
+      <c r="H28" s="77"/>
     </row>
     <row r="29" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="30" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B30" s="84" t="s">
+      <c r="B30" s="81" t="s">
         <v>15</v>
       </c>
-      <c r="C30" s="76"/>
-      <c r="D30" s="76"/>
-      <c r="E30" s="76"/>
-      <c r="F30" s="76"/>
-      <c r="G30" s="76"/>
-      <c r="H30" s="76"/>
+      <c r="C30" s="77"/>
+      <c r="D30" s="77"/>
+      <c r="E30" s="77"/>
+      <c r="F30" s="77"/>
+      <c r="G30" s="77"/>
+      <c r="H30" s="77"/>
     </row>
     <row r="31" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B31" s="82" t="s">
+      <c r="B31" s="79" t="s">
         <v>16</v>
       </c>
-      <c r="C31" s="76"/>
-      <c r="D31" s="76"/>
-      <c r="E31" s="76"/>
-      <c r="F31" s="76"/>
-      <c r="G31" s="76"/>
-      <c r="H31" s="76"/>
+      <c r="C31" s="77"/>
+      <c r="D31" s="77"/>
+      <c r="E31" s="77"/>
+      <c r="F31" s="77"/>
+      <c r="G31" s="77"/>
+      <c r="H31" s="77"/>
     </row>
     <row r="32" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="33" spans="2:8" ht="18" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="34" spans="2:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="87" t="s">
+      <c r="B34" s="84" t="s">
         <v>17</v>
       </c>
-      <c r="C34" s="76"/>
-      <c r="D34" s="76"/>
-      <c r="E34" s="76"/>
-      <c r="F34" s="76"/>
-      <c r="G34" s="76"/>
-      <c r="H34" s="76"/>
+      <c r="C34" s="77"/>
+      <c r="D34" s="77"/>
+      <c r="E34" s="77"/>
+      <c r="F34" s="77"/>
+      <c r="G34" s="77"/>
+      <c r="H34" s="77"/>
     </row>
     <row r="35" spans="2:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="85" t="s">
+      <c r="B35" s="82" t="s">
         <v>18</v>
       </c>
-      <c r="C35" s="76"/>
-      <c r="D35" s="76"/>
-      <c r="E35" s="76"/>
-      <c r="F35" s="76"/>
-      <c r="G35" s="76"/>
-      <c r="H35" s="76"/>
+      <c r="C35" s="77"/>
+      <c r="D35" s="77"/>
+      <c r="E35" s="77"/>
+      <c r="F35" s="77"/>
+      <c r="G35" s="77"/>
+      <c r="H35" s="77"/>
     </row>
     <row r="36" spans="2:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B36" s="85" t="s">
+      <c r="B36" s="82" t="s">
         <v>19</v>
       </c>
-      <c r="C36" s="76"/>
-      <c r="D36" s="76"/>
-      <c r="E36" s="76"/>
-      <c r="F36" s="76"/>
-      <c r="G36" s="76"/>
-      <c r="H36" s="76"/>
+      <c r="C36" s="77"/>
+      <c r="D36" s="77"/>
+      <c r="E36" s="77"/>
+      <c r="F36" s="77"/>
+      <c r="G36" s="77"/>
+      <c r="H36" s="77"/>
     </row>
     <row r="37" spans="2:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B37" s="85" t="s">
+      <c r="B37" s="82" t="s">
         <v>20</v>
       </c>
-      <c r="C37" s="76"/>
-      <c r="D37" s="76"/>
-      <c r="E37" s="76"/>
-      <c r="F37" s="76"/>
-      <c r="G37" s="76"/>
-      <c r="H37" s="76"/>
+      <c r="C37" s="77"/>
+      <c r="D37" s="77"/>
+      <c r="E37" s="77"/>
+      <c r="F37" s="77"/>
+      <c r="G37" s="77"/>
+      <c r="H37" s="77"/>
     </row>
     <row r="38" spans="2:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B38" s="85" t="s">
+      <c r="B38" s="82" t="s">
         <v>21</v>
       </c>
-      <c r="C38" s="76"/>
-      <c r="D38" s="76"/>
-      <c r="E38" s="76"/>
-      <c r="F38" s="76"/>
-      <c r="G38" s="76"/>
-      <c r="H38" s="76"/>
+      <c r="C38" s="77"/>
+      <c r="D38" s="77"/>
+      <c r="E38" s="77"/>
+      <c r="F38" s="77"/>
+      <c r="G38" s="77"/>
+      <c r="H38" s="77"/>
     </row>
     <row r="39" spans="2:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B39" s="85" t="s">
+      <c r="B39" s="82" t="s">
         <v>22</v>
       </c>
-      <c r="C39" s="76"/>
-      <c r="D39" s="76"/>
-      <c r="E39" s="76"/>
-      <c r="F39" s="76"/>
-      <c r="G39" s="76"/>
-      <c r="H39" s="76"/>
+      <c r="C39" s="77"/>
+      <c r="D39" s="77"/>
+      <c r="E39" s="77"/>
+      <c r="F39" s="77"/>
+      <c r="G39" s="77"/>
+      <c r="H39" s="77"/>
     </row>
   </sheetData>
   <mergeCells count="23">
@@ -7650,34 +7672,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="80" t="s">
+      <c r="A1" s="76" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="80"/>
-      <c r="C1" s="80"/>
-      <c r="D1" s="80"/>
-      <c r="E1" s="80"/>
-      <c r="F1" s="80"/>
-      <c r="G1" s="80"/>
-      <c r="H1" s="80"/>
-      <c r="I1" s="80"/>
-      <c r="J1" s="80"/>
-      <c r="K1" s="80"/>
+      <c r="B1" s="76"/>
+      <c r="C1" s="76"/>
+      <c r="D1" s="76"/>
+      <c r="E1" s="76"/>
+      <c r="F1" s="76"/>
+      <c r="G1" s="76"/>
+      <c r="H1" s="76"/>
+      <c r="I1" s="76"/>
+      <c r="J1" s="76"/>
+      <c r="K1" s="76"/>
     </row>
     <row r="2" spans="1:11" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="79" t="s">
+      <c r="A2" s="88" t="s">
         <v>24</v>
       </c>
-      <c r="B2" s="79"/>
-      <c r="C2" s="79"/>
-      <c r="D2" s="79"/>
-      <c r="E2" s="79"/>
-      <c r="F2" s="79"/>
-      <c r="G2" s="79"/>
-      <c r="H2" s="79"/>
-      <c r="I2" s="79"/>
-      <c r="J2" s="79"/>
-      <c r="K2" s="79"/>
+      <c r="B2" s="88"/>
+      <c r="C2" s="88"/>
+      <c r="D2" s="88"/>
+      <c r="E2" s="88"/>
+      <c r="F2" s="88"/>
+      <c r="G2" s="88"/>
+      <c r="H2" s="88"/>
+      <c r="I2" s="88"/>
+      <c r="J2" s="88"/>
+      <c r="K2" s="88"/>
     </row>
     <row r="3" spans="1:11" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
@@ -8199,10 +8221,10 @@
       </c>
     </row>
     <row r="15" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="77" t="s">
+      <c r="A15" s="86" t="s">
         <v>36</v>
       </c>
-      <c r="B15" s="78"/>
+      <c r="B15" s="87"/>
       <c r="C15" s="16">
         <f>+SUM(C4:C14)</f>
         <v>131513.58530100001</v>
@@ -8239,34 +8261,34 @@
     </row>
     <row r="16" spans="1:11" ht="10.050000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="17" spans="1:11" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="80" t="s">
+      <c r="A17" s="76" t="s">
         <v>38</v>
       </c>
-      <c r="B17" s="76"/>
-      <c r="C17" s="76"/>
-      <c r="D17" s="76"/>
-      <c r="E17" s="76"/>
-      <c r="F17" s="76"/>
-      <c r="G17" s="76"/>
-      <c r="H17" s="76"/>
-      <c r="I17" s="76"/>
-      <c r="J17" s="76"/>
-      <c r="K17" s="76"/>
+      <c r="B17" s="77"/>
+      <c r="C17" s="77"/>
+      <c r="D17" s="77"/>
+      <c r="E17" s="77"/>
+      <c r="F17" s="77"/>
+      <c r="G17" s="77"/>
+      <c r="H17" s="77"/>
+      <c r="I17" s="77"/>
+      <c r="J17" s="77"/>
+      <c r="K17" s="77"/>
     </row>
     <row r="18" spans="1:11" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="75" t="s">
+      <c r="A18" s="85" t="s">
         <v>39</v>
       </c>
-      <c r="B18" s="76"/>
-      <c r="C18" s="76"/>
-      <c r="D18" s="76"/>
-      <c r="E18" s="76"/>
-      <c r="F18" s="76"/>
-      <c r="G18" s="76"/>
-      <c r="H18" s="76"/>
-      <c r="I18" s="76"/>
-      <c r="J18" s="76"/>
-      <c r="K18" s="76"/>
+      <c r="B18" s="77"/>
+      <c r="C18" s="77"/>
+      <c r="D18" s="77"/>
+      <c r="E18" s="77"/>
+      <c r="F18" s="77"/>
+      <c r="G18" s="77"/>
+      <c r="H18" s="77"/>
+      <c r="I18" s="77"/>
+      <c r="J18" s="77"/>
+      <c r="K18" s="77"/>
     </row>
     <row r="19" spans="1:11" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="3" t="s">
@@ -8658,10 +8680,10 @@
       </c>
     </row>
     <row r="31" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="77" t="s">
+      <c r="A31" s="86" t="s">
         <v>36</v>
       </c>
-      <c r="B31" s="78"/>
+      <c r="B31" s="87"/>
       <c r="C31" s="16">
         <f>+SUM(C20:C30)</f>
         <v>613245.82780000009</v>
@@ -8718,34 +8740,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="91" t="s">
+      <c r="A1" s="92" t="s">
         <v>2019</v>
       </c>
-      <c r="B1" s="76"/>
-      <c r="C1" s="76"/>
-      <c r="D1" s="76"/>
-      <c r="E1" s="76"/>
-      <c r="F1" s="76"/>
-      <c r="G1" s="76"/>
-      <c r="H1" s="76"/>
-      <c r="I1" s="76"/>
-      <c r="J1" s="76"/>
-      <c r="K1" s="76"/>
+      <c r="B1" s="77"/>
+      <c r="C1" s="77"/>
+      <c r="D1" s="77"/>
+      <c r="E1" s="77"/>
+      <c r="F1" s="77"/>
+      <c r="G1" s="77"/>
+      <c r="H1" s="77"/>
+      <c r="I1" s="77"/>
+      <c r="J1" s="77"/>
+      <c r="K1" s="77"/>
     </row>
     <row r="2" spans="1:11" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="90" t="s">
+      <c r="A2" s="91" t="s">
         <v>46</v>
       </c>
-      <c r="B2" s="76"/>
-      <c r="C2" s="76"/>
-      <c r="D2" s="76"/>
-      <c r="E2" s="76"/>
-      <c r="F2" s="76"/>
-      <c r="G2" s="76"/>
-      <c r="H2" s="76"/>
-      <c r="I2" s="76"/>
-      <c r="J2" s="76"/>
-      <c r="K2" s="76"/>
+      <c r="B2" s="77"/>
+      <c r="C2" s="77"/>
+      <c r="D2" s="77"/>
+      <c r="E2" s="77"/>
+      <c r="F2" s="77"/>
+      <c r="G2" s="77"/>
+      <c r="H2" s="77"/>
+      <c r="I2" s="77"/>
+      <c r="J2" s="77"/>
+      <c r="K2" s="77"/>
     </row>
     <row r="3" spans="1:11" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="20" t="s">
@@ -9355,10 +9377,10 @@
       </c>
     </row>
     <row r="17" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="92" t="s">
+      <c r="A17" s="93" t="s">
         <v>36</v>
       </c>
-      <c r="B17" s="78"/>
+      <c r="B17" s="87"/>
       <c r="C17" s="21">
         <f>+SUM(C4:C16)</f>
         <v>3882791</v>
@@ -9392,34 +9414,34 @@
       <c r="K17" s="56"/>
     </row>
     <row r="21" spans="1:11" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A21" s="91" t="s">
+      <c r="A21" s="92" t="s">
         <v>38</v>
       </c>
-      <c r="B21" s="76"/>
-      <c r="C21" s="76"/>
-      <c r="D21" s="76"/>
-      <c r="E21" s="76"/>
-      <c r="F21" s="76"/>
-      <c r="G21" s="76"/>
-      <c r="H21" s="76"/>
-      <c r="I21" s="76"/>
-      <c r="J21" s="76"/>
-      <c r="K21" s="76"/>
+      <c r="B21" s="77"/>
+      <c r="C21" s="77"/>
+      <c r="D21" s="77"/>
+      <c r="E21" s="77"/>
+      <c r="F21" s="77"/>
+      <c r="G21" s="77"/>
+      <c r="H21" s="77"/>
+      <c r="I21" s="77"/>
+      <c r="J21" s="77"/>
+      <c r="K21" s="77"/>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A22" s="90" t="s">
+      <c r="A22" s="91" t="s">
         <v>39</v>
       </c>
-      <c r="B22" s="76"/>
-      <c r="C22" s="76"/>
-      <c r="D22" s="76"/>
-      <c r="E22" s="76"/>
-      <c r="F22" s="76"/>
-      <c r="G22" s="76"/>
-      <c r="H22" s="76"/>
-      <c r="I22" s="76"/>
-      <c r="J22" s="76"/>
-      <c r="K22" s="76"/>
+      <c r="B22" s="77"/>
+      <c r="C22" s="77"/>
+      <c r="D22" s="77"/>
+      <c r="E22" s="77"/>
+      <c r="F22" s="77"/>
+      <c r="G22" s="77"/>
+      <c r="H22" s="77"/>
+      <c r="I22" s="77"/>
+      <c r="J22" s="77"/>
+      <c r="K22" s="77"/>
     </row>
     <row r="23" spans="1:11" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A23" s="20" t="s">
@@ -9877,10 +9899,10 @@
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A37" s="88" t="s">
+      <c r="A37" s="89" t="s">
         <v>36</v>
       </c>
-      <c r="B37" s="89"/>
+      <c r="B37" s="90"/>
       <c r="C37" s="21">
         <f>+SUM(C24:C36)</f>
         <v>32689269.600000001</v>
@@ -9937,34 +9959,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="91" t="s">
+      <c r="A1" s="92" t="s">
         <v>2021</v>
       </c>
-      <c r="B1" s="76"/>
-      <c r="C1" s="76"/>
-      <c r="D1" s="76"/>
-      <c r="E1" s="76"/>
-      <c r="F1" s="76"/>
-      <c r="G1" s="76"/>
-      <c r="H1" s="76"/>
-      <c r="I1" s="76"/>
-      <c r="J1" s="76"/>
-      <c r="K1" s="76"/>
+      <c r="B1" s="77"/>
+      <c r="C1" s="77"/>
+      <c r="D1" s="77"/>
+      <c r="E1" s="77"/>
+      <c r="F1" s="77"/>
+      <c r="G1" s="77"/>
+      <c r="H1" s="77"/>
+      <c r="I1" s="77"/>
+      <c r="J1" s="77"/>
+      <c r="K1" s="77"/>
     </row>
     <row r="2" spans="1:11" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="93" t="s">
+      <c r="A2" s="94" t="s">
         <v>46</v>
       </c>
-      <c r="B2" s="94"/>
-      <c r="C2" s="94"/>
-      <c r="D2" s="94"/>
-      <c r="E2" s="94"/>
-      <c r="F2" s="94"/>
-      <c r="G2" s="94"/>
-      <c r="H2" s="94"/>
-      <c r="I2" s="94"/>
-      <c r="J2" s="94"/>
-      <c r="K2" s="94"/>
+      <c r="B2" s="95"/>
+      <c r="C2" s="95"/>
+      <c r="D2" s="95"/>
+      <c r="E2" s="95"/>
+      <c r="F2" s="95"/>
+      <c r="G2" s="95"/>
+      <c r="H2" s="95"/>
+      <c r="I2" s="95"/>
+      <c r="J2" s="95"/>
+      <c r="K2" s="95"/>
     </row>
     <row r="3" spans="1:11" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="20" t="s">
@@ -10573,10 +10595,10 @@
       </c>
     </row>
     <row r="17" spans="1:11" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="95" t="s">
+      <c r="A17" s="96" t="s">
         <v>36</v>
       </c>
-      <c r="B17" s="78"/>
+      <c r="B17" s="87"/>
       <c r="C17" s="21">
         <f>+SUM(C4:C16)</f>
         <v>4145818.1706020003</v>
@@ -10610,34 +10632,34 @@
       <c r="K17" s="56"/>
     </row>
     <row r="20" spans="1:11" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A20" s="91" t="s">
+      <c r="A20" s="92" t="s">
         <v>2020</v>
       </c>
-      <c r="B20" s="76"/>
-      <c r="C20" s="76"/>
-      <c r="D20" s="76"/>
-      <c r="E20" s="76"/>
-      <c r="F20" s="76"/>
-      <c r="G20" s="76"/>
-      <c r="H20" s="76"/>
-      <c r="I20" s="76"/>
-      <c r="J20" s="76"/>
-      <c r="K20" s="76"/>
+      <c r="B20" s="77"/>
+      <c r="C20" s="77"/>
+      <c r="D20" s="77"/>
+      <c r="E20" s="77"/>
+      <c r="F20" s="77"/>
+      <c r="G20" s="77"/>
+      <c r="H20" s="77"/>
+      <c r="I20" s="77"/>
+      <c r="J20" s="77"/>
+      <c r="K20" s="77"/>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A21" s="90" t="s">
+      <c r="A21" s="91" t="s">
         <v>39</v>
       </c>
-      <c r="B21" s="76"/>
-      <c r="C21" s="76"/>
-      <c r="D21" s="76"/>
-      <c r="E21" s="76"/>
-      <c r="F21" s="76"/>
-      <c r="G21" s="76"/>
-      <c r="H21" s="76"/>
-      <c r="I21" s="76"/>
-      <c r="J21" s="76"/>
-      <c r="K21" s="76"/>
+      <c r="B21" s="77"/>
+      <c r="C21" s="77"/>
+      <c r="D21" s="77"/>
+      <c r="E21" s="77"/>
+      <c r="F21" s="77"/>
+      <c r="G21" s="77"/>
+      <c r="H21" s="77"/>
+      <c r="I21" s="77"/>
+      <c r="J21" s="77"/>
+      <c r="K21" s="77"/>
     </row>
     <row r="22" spans="1:11" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A22" s="20" t="s">
@@ -11095,10 +11117,10 @@
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A36" s="88" t="s">
+      <c r="A36" s="89" t="s">
         <v>36</v>
       </c>
-      <c r="B36" s="89"/>
+      <c r="B36" s="90"/>
       <c r="C36" s="21">
         <f>+SUM(C23:C35)</f>
         <v>33302515.427800003</v>
@@ -11137,7 +11159,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <sheetPr filterMode="1">
+  <sheetPr>
     <tabColor rgb="FF2E5FA3"/>
   </sheetPr>
   <dimension ref="A1:P136"/>
@@ -11153,23 +11175,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="80" t="s">
+      <c r="A1" s="76" t="s">
         <v>56</v>
       </c>
-      <c r="B1" s="76"/>
-      <c r="C1" s="76"/>
-      <c r="D1" s="76"/>
-      <c r="E1" s="76"/>
-      <c r="F1" s="76"/>
-      <c r="G1" s="76"/>
-      <c r="H1" s="76"/>
-      <c r="I1" s="76"/>
-      <c r="J1" s="76"/>
-      <c r="K1" s="76"/>
-      <c r="L1" s="76"/>
-      <c r="M1" s="76"/>
-      <c r="N1" s="76"/>
-      <c r="O1" s="76"/>
+      <c r="B1" s="77"/>
+      <c r="C1" s="77"/>
+      <c r="D1" s="77"/>
+      <c r="E1" s="77"/>
+      <c r="F1" s="77"/>
+      <c r="G1" s="77"/>
+      <c r="H1" s="77"/>
+      <c r="I1" s="77"/>
+      <c r="J1" s="77"/>
+      <c r="K1" s="77"/>
+      <c r="L1" s="77"/>
+      <c r="M1" s="77"/>
+      <c r="N1" s="77"/>
+      <c r="O1" s="77"/>
     </row>
     <row r="2" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="25" t="s">
@@ -11221,7 +11243,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="3" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="30" t="s">
         <v>61</v>
       </c>
@@ -11275,7 +11297,7 @@
         <v>3.9015900423134818E-4</v>
       </c>
     </row>
-    <row r="4" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="26" t="s">
         <v>61</v>
       </c>
@@ -11321,7 +11343,7 @@
         <v>3.9969675920259814E-4</v>
       </c>
     </row>
-    <row r="5" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="26" t="s">
         <v>61</v>
       </c>
@@ -11421,7 +11443,7 @@
         <v>3.3700640872303105E-4</v>
       </c>
     </row>
-    <row r="7" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="30" t="s">
         <v>61</v>
       </c>
@@ -11467,7 +11489,7 @@
         <v>1.3703268103059283E-3</v>
       </c>
     </row>
-    <row r="8" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="30" t="s">
         <v>61</v>
       </c>
@@ -11567,7 +11589,7 @@
         <v>1.2160098195280687E-4</v>
       </c>
     </row>
-    <row r="10" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="26" t="s">
         <v>61</v>
       </c>
@@ -11621,7 +11643,7 @@
         <v>6.8937346328444893E-5</v>
       </c>
     </row>
-    <row r="11" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="30" t="s">
         <v>61</v>
       </c>
@@ -11675,7 +11697,7 @@
         <v>6.960319939146195E-5</v>
       </c>
     </row>
-    <row r="12" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="30" t="s">
         <v>61</v>
       </c>
@@ -11729,7 +11751,7 @@
         <v>6.7237487425238213E-5</v>
       </c>
     </row>
-    <row r="13" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="26" t="s">
         <v>61</v>
       </c>
@@ -11783,7 +11805,7 @@
         <v>1.0046147155141154E-4</v>
       </c>
     </row>
-    <row r="14" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="30" t="s">
         <v>61</v>
       </c>
@@ -11837,7 +11859,7 @@
         <v>7.6331834535891413E-5</v>
       </c>
     </row>
-    <row r="15" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="26" t="s">
         <v>61</v>
       </c>
@@ -11891,7 +11913,7 @@
         <v>8.2821364680362336E-5</v>
       </c>
     </row>
-    <row r="16" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="30" t="s">
         <v>61</v>
       </c>
@@ -11945,7 +11967,7 @@
         <v>8.6796790177445489E-5</v>
       </c>
     </row>
-    <row r="17" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="30" t="s">
         <v>61</v>
       </c>
@@ -12045,7 +12067,7 @@
         <v>8.3843321475597177E-5</v>
       </c>
     </row>
-    <row r="19" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="26" t="s">
         <v>61</v>
       </c>
@@ -12089,7 +12111,7 @@
         <v>4.4033508724473609E-7</v>
       </c>
     </row>
-    <row r="20" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="26" t="s">
         <v>61</v>
       </c>
@@ -12143,7 +12165,7 @@
         <v>6.9188193220106952E-7</v>
       </c>
     </row>
-    <row r="21" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="26" t="s">
         <v>61</v>
       </c>
@@ -12251,7 +12273,7 @@
         <v>1.6421973545855717E-6</v>
       </c>
     </row>
-    <row r="23" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="30" t="s">
         <v>61</v>
       </c>
@@ -12305,7 +12327,7 @@
         <v>3.4674789373453067E-4</v>
       </c>
     </row>
-    <row r="24" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="30" t="s">
         <v>61</v>
       </c>
@@ -12359,7 +12381,7 @@
         <v>3.2142895495218749E-4</v>
       </c>
     </row>
-    <row r="25" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="30" t="s">
         <v>61</v>
       </c>
@@ -12413,7 +12435,7 @@
         <v>2.904547532167844E-4</v>
       </c>
     </row>
-    <row r="26" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="30" t="s">
         <v>61</v>
       </c>
@@ -12467,7 +12489,7 @@
         <v>3.5158149562828473E-4</v>
       </c>
     </row>
-    <row r="27" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="30" t="s">
         <v>61</v>
       </c>
@@ -12521,7 +12543,7 @@
         <v>3.8390391971499172E-4</v>
       </c>
     </row>
-    <row r="28" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="26" t="s">
         <v>61</v>
       </c>
@@ -12575,7 +12597,7 @@
         <v>8.0105649320888012E-5</v>
       </c>
     </row>
-    <row r="29" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="26" t="s">
         <v>61</v>
       </c>
@@ -12629,7 +12651,7 @@
         <v>6.1749551470887803E-5</v>
       </c>
     </row>
-    <row r="30" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="26" t="s">
         <v>61</v>
       </c>
@@ -12683,7 +12705,7 @@
         <v>1.2085936408953657E-4</v>
       </c>
     </row>
-    <row r="31" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="26" t="s">
         <v>61</v>
       </c>
@@ -12791,7 +12813,7 @@
         <v>1.0032778704175664E-4</v>
       </c>
     </row>
-    <row r="33" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="30" t="s">
         <v>61</v>
       </c>
@@ -12845,7 +12867,7 @@
         <v>1.9619966759802478E-5</v>
       </c>
     </row>
-    <row r="34" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="30" t="s">
         <v>61</v>
       </c>
@@ -12897,7 +12919,7 @@
         <v>1.2853243888531356E-4</v>
       </c>
     </row>
-    <row r="35" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="30" t="s">
         <v>61</v>
       </c>
@@ -12949,7 +12971,7 @@
         <v>9.0417087058252167E-5</v>
       </c>
     </row>
-    <row r="36" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="26" t="s">
         <v>61</v>
       </c>
@@ -12997,7 +13019,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="26" t="s">
         <v>61</v>
       </c>
@@ -13045,7 +13067,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="26" t="s">
         <v>61</v>
       </c>
@@ -13097,7 +13119,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="30" t="s">
         <v>61</v>
       </c>
@@ -13149,7 +13171,7 @@
         <v>8.0803389328355983E-10</v>
       </c>
     </row>
-    <row r="40" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="30" t="s">
         <v>61</v>
       </c>
@@ -13197,7 +13219,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="30" t="s">
         <v>61</v>
       </c>
@@ -13245,7 +13267,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="26" t="s">
         <v>61</v>
       </c>
@@ -13299,7 +13321,7 @@
         <v>3.1423482925962134E-7</v>
       </c>
     </row>
-    <row r="43" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="26" t="s">
         <v>61</v>
       </c>
@@ -13351,7 +13373,7 @@
         <v>4.0279830064411784E-4</v>
       </c>
     </row>
-    <row r="44" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="26" t="s">
         <v>61</v>
       </c>
@@ -13403,7 +13425,7 @@
         <v>4.105507252619632E-4</v>
       </c>
     </row>
-    <row r="45" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="26" t="s">
         <v>61</v>
       </c>
@@ -13457,7 +13479,7 @@
         <v>2.5024382110745187E-4</v>
       </c>
     </row>
-    <row r="46" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="30" t="s">
         <v>61</v>
       </c>
@@ -13511,7 +13533,7 @@
         <v>2.0964689752467623E-4</v>
       </c>
     </row>
-    <row r="47" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="30" t="s">
         <v>61</v>
       </c>
@@ -13565,7 +13587,7 @@
         <v>1.7717053682646228E-4</v>
       </c>
     </row>
-    <row r="48" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="30" t="s">
         <v>61</v>
       </c>
@@ -13619,7 +13641,7 @@
         <v>2.6061269851365639E-4</v>
       </c>
     </row>
-    <row r="49" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A49" s="26" t="s">
         <v>61</v>
       </c>
@@ -13673,7 +13695,7 @@
         <v>2.802082543743464E-4</v>
       </c>
     </row>
-    <row r="50" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50" s="30" t="s">
         <v>61</v>
       </c>
@@ -13727,7 +13749,7 @@
         <v>1.3218694624976203E-3</v>
       </c>
     </row>
-    <row r="51" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" s="26" t="s">
         <v>61</v>
       </c>
@@ -13771,7 +13793,7 @@
         <v>2.1699947493818676E-4</v>
       </c>
     </row>
-    <row r="52" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="30" t="s">
         <v>61</v>
       </c>
@@ -13815,7 +13837,7 @@
         <v>2.0678091880093621E-4</v>
       </c>
     </row>
-    <row r="53" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" s="30" t="s">
         <v>61</v>
       </c>
@@ -13859,7 +13881,7 @@
         <v>2.2159758133251538E-4</v>
       </c>
     </row>
-    <row r="54" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" s="30" t="s">
         <v>61</v>
       </c>
@@ -13913,7 +13935,7 @@
         <v>2.1592227991997255E-4</v>
       </c>
     </row>
-    <row r="55" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A55" s="30" t="s">
         <v>61</v>
       </c>
@@ -13967,7 +13989,7 @@
         <v>2.4123316060138688E-4</v>
       </c>
     </row>
-    <row r="56" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A56" s="26" t="s">
         <v>61</v>
       </c>
@@ -14013,7 +14035,7 @@
         <v>2.2925214853761495E-4</v>
       </c>
     </row>
-    <row r="57" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A57" s="30" t="s">
         <v>61</v>
       </c>
@@ -14067,7 +14089,7 @@
         <v>1.1999918163111271E-3</v>
       </c>
     </row>
-    <row r="58" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A58" s="26" t="s">
         <v>61</v>
       </c>
@@ -14119,7 +14141,7 @@
         <v>1.1999918163111271E-3</v>
       </c>
     </row>
-    <row r="59" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A59" s="26" t="s">
         <v>61</v>
       </c>
@@ -14173,7 +14195,7 @@
         <v>5.157181358694042E-8</v>
       </c>
     </row>
-    <row r="60" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A60" s="26" t="s">
         <v>61</v>
       </c>
@@ -14227,7 +14249,7 @@
         <v>4.5597312439003996E-8</v>
       </c>
     </row>
-    <row r="61" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A61" s="26" t="s">
         <v>61</v>
       </c>
@@ -14279,7 +14301,7 @@
         <v>1.062953370580349E-4</v>
       </c>
     </row>
-    <row r="62" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A62" s="30" t="s">
         <v>61</v>
       </c>
@@ -14331,7 +14353,7 @@
         <v>9.880242995883322E-5</v>
       </c>
     </row>
-    <row r="63" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A63" s="30" t="s">
         <v>61</v>
       </c>
@@ -14383,7 +14405,7 @@
         <v>8.6951812159156213E-5</v>
       </c>
     </row>
-    <row r="64" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A64" s="30" t="s">
         <v>61</v>
       </c>
@@ -14437,7 +14459,7 @@
         <v>7.9050766973426647E-5</v>
       </c>
     </row>
-    <row r="65" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A65" s="26" t="s">
         <v>61</v>
       </c>
@@ -14491,7 +14513,7 @@
         <v>7.4440071337186902E-5</v>
       </c>
     </row>
-    <row r="66" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A66" s="30" t="s">
         <v>61</v>
       </c>
@@ -14541,7 +14563,7 @@
         <v>4.922576828981495E-5</v>
       </c>
     </row>
-    <row r="67" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A67" s="30" t="s">
         <v>61</v>
       </c>
@@ -14591,7 +14613,7 @@
         <v>5.72542447631843E-5</v>
       </c>
     </row>
-    <row r="68" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A68" s="26" t="s">
         <v>61</v>
       </c>
@@ -14645,7 +14667,7 @@
         <v>7.6612693911474235E-4</v>
       </c>
     </row>
-    <row r="69" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A69" s="30" t="s">
         <v>61</v>
       </c>
@@ -14699,7 +14721,7 @@
         <v>7.2904093800786553E-4</v>
       </c>
     </row>
-    <row r="70" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A70" s="26" t="s">
         <v>61</v>
       </c>
@@ -14753,7 +14775,7 @@
         <v>9.3328716206789023E-5</v>
       </c>
     </row>
-    <row r="71" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A71" s="26" t="s">
         <v>61</v>
       </c>
@@ -14807,7 +14829,7 @@
         <v>7.2219831218339785E-5</v>
       </c>
     </row>
-    <row r="72" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A72" s="30" t="s">
         <v>61</v>
       </c>
@@ -14861,7 +14883,7 @@
         <v>1.4722553282300169E-6</v>
       </c>
     </row>
-    <row r="73" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A73" s="26" t="s">
         <v>61</v>
       </c>
@@ -14915,7 +14937,7 @@
         <v>1.8061457910467699E-6</v>
       </c>
     </row>
-    <row r="74" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A74" s="30" t="s">
         <v>61</v>
       </c>
@@ -14969,7 +14991,7 @@
         <v>1.7438959027054161E-6</v>
       </c>
     </row>
-    <row r="75" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A75" s="26" t="s">
         <v>61</v>
       </c>
@@ -15077,7 +15099,7 @@
         <v>2.1583447531068846E-3</v>
       </c>
     </row>
-    <row r="77" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A77" s="30" t="s">
         <v>61</v>
       </c>
@@ -15131,7 +15153,7 @@
         <v>2.0834075775478912E-4</v>
       </c>
     </row>
-    <row r="78" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A78" s="26" t="s">
         <v>61</v>
       </c>
@@ -15185,7 +15207,7 @@
         <v>1.9571940952326655E-4</v>
       </c>
     </row>
-    <row r="79" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A79" s="30" t="s">
         <v>61</v>
       </c>
@@ -15239,7 +15261,7 @@
         <v>1.3204367698076472E-4</v>
       </c>
     </row>
-    <row r="80" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A80" s="30" t="s">
         <v>61</v>
       </c>
@@ -15347,7 +15369,7 @@
         <v>1.5582207937015781E-4</v>
       </c>
     </row>
-    <row r="82" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A82" s="26" t="s">
         <v>61</v>
       </c>
@@ -15401,7 +15423,7 @@
         <v>6.960319939146195E-5</v>
       </c>
     </row>
-    <row r="83" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A83" s="30" t="s">
         <v>61</v>
       </c>
@@ -15455,7 +15477,7 @@
         <v>6.7237487425238213E-5</v>
       </c>
     </row>
-    <row r="84" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A84" s="26" t="s">
         <v>61</v>
       </c>
@@ -15509,7 +15531,7 @@
         <v>1.6018857928033528E-4</v>
       </c>
     </row>
-    <row r="85" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A85" s="26" t="s">
         <v>61</v>
       </c>
@@ -15563,7 +15585,7 @@
         <v>2.1478820228937383E-4</v>
       </c>
     </row>
-    <row r="86" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A86" s="30" t="s">
         <v>61</v>
       </c>
@@ -15617,7 +15639,7 @@
         <v>6.7998839778333857E-4</v>
       </c>
     </row>
-    <row r="87" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A87" s="26" t="s">
         <v>61</v>
       </c>
@@ -15725,7 +15747,7 @@
         <v>3.1680449062079753E-4</v>
       </c>
     </row>
-    <row r="89" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A89" s="30" t="s">
         <v>61</v>
       </c>
@@ -15779,7 +15801,7 @@
         <v>3.2670430030544692E-7</v>
       </c>
     </row>
-    <row r="90" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A90" s="26" t="s">
         <v>61</v>
       </c>
@@ -15833,7 +15855,7 @@
         <v>7.0104731828297285E-6</v>
       </c>
     </row>
-    <row r="91" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A91" s="26" t="s">
         <v>61</v>
       </c>
@@ -15879,7 +15901,7 @@
         <v>1.680254517607324E-5</v>
       </c>
     </row>
-    <row r="92" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A92" s="30" t="s">
         <v>61</v>
       </c>
@@ -15925,7 +15947,7 @@
         <v>2.1502222166801437E-5</v>
       </c>
     </row>
-    <row r="93" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A93" s="30" t="s">
         <v>61</v>
       </c>
@@ -16033,7 +16055,7 @@
         <v>1.0506816014110938E-4</v>
       </c>
     </row>
-    <row r="95" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A95" s="26" t="s">
         <v>61</v>
       </c>
@@ -16087,7 +16109,7 @@
         <v>9.4819491641413156E-5</v>
       </c>
     </row>
-    <row r="96" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A96" s="26" t="s">
         <v>61</v>
       </c>
@@ -16195,7 +16217,7 @@
         <v>1.4470728881392812E-4</v>
       </c>
     </row>
-    <row r="98" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A98" s="26" t="s">
         <v>61</v>
       </c>
@@ -16249,7 +16271,7 @@
         <v>1.0126982067727716E-7</v>
       </c>
     </row>
-    <row r="99" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A99" s="26" t="s">
         <v>61</v>
       </c>
@@ -16303,7 +16325,7 @@
         <v>1.1180907316873605E-7</v>
       </c>
     </row>
-    <row r="100" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A100" s="26" t="s">
         <v>61</v>
       </c>
@@ -16357,7 +16379,7 @@
         <v>7.5689308767206315E-8</v>
       </c>
     </row>
-    <row r="101" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A101" s="30" t="s">
         <v>61</v>
       </c>
@@ -16409,7 +16431,7 @@
         <v>6.7898748685067387E-8</v>
       </c>
     </row>
-    <row r="102" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A102" s="26" t="s">
         <v>61</v>
       </c>
@@ -16461,7 +16483,7 @@
         <v>1.4462490808278257E-4</v>
       </c>
     </row>
-    <row r="103" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A103" s="30" t="s">
         <v>61</v>
       </c>
@@ -16513,7 +16535,7 @@
         <v>9.9049581952307192E-5</v>
       </c>
     </row>
-    <row r="104" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A104" s="30" t="s">
         <v>61</v>
       </c>
@@ -16567,7 +16589,7 @@
         <v>3.3319462408952943E-5</v>
       </c>
     </row>
-    <row r="105" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A105" s="26" t="s">
         <v>61</v>
       </c>
@@ -16617,7 +16639,7 @@
         <v>8.5996969197540062E-4</v>
       </c>
     </row>
-    <row r="106" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A106" s="30" t="s">
         <v>61</v>
       </c>
@@ -16671,7 +16693,7 @@
         <v>6.2283265692645857E-4</v>
       </c>
     </row>
-    <row r="107" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A107" s="26" t="s">
         <v>61</v>
       </c>
@@ -16779,7 +16801,7 @@
         <v>1.9422554928817665E-5</v>
       </c>
     </row>
-    <row r="109" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A109" s="26" t="s">
         <v>61</v>
       </c>
@@ -16833,7 +16855,7 @@
         <v>8.7996404629767452E-5</v>
       </c>
     </row>
-    <row r="110" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A110" s="30" t="s">
         <v>61</v>
       </c>
@@ -16887,7 +16909,7 @@
         <v>8.8223579610939511E-5</v>
       </c>
     </row>
-    <row r="111" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A111" s="26" t="s">
         <v>61</v>
       </c>
@@ -16941,7 +16963,7 @@
         <v>9.1421666142160981E-5</v>
       </c>
     </row>
-    <row r="112" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A112" s="30" t="s">
         <v>61</v>
       </c>
@@ -16995,7 +17017,7 @@
         <v>8.3559988063918245E-5</v>
       </c>
     </row>
-    <row r="113" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A113" s="26" t="s">
         <v>61</v>
       </c>
@@ -17049,7 +17071,7 @@
         <v>8.6832207855670567E-5</v>
       </c>
     </row>
-    <row r="114" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A114" s="30" t="s">
         <v>61</v>
       </c>
@@ -17157,7 +17179,7 @@
         <v>8.8641315872164708E-5</v>
       </c>
     </row>
-    <row r="116" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A116" s="30" t="s">
         <v>61</v>
       </c>
@@ -17201,7 +17223,7 @@
         <v>1.1534143585270261E-4</v>
       </c>
     </row>
-    <row r="117" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A117" s="26" t="s">
         <v>61</v>
       </c>
@@ -17245,7 +17267,7 @@
         <v>1.1589731845046669E-4</v>
       </c>
     </row>
-    <row r="118" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A118" s="30" t="s">
         <v>61</v>
       </c>
@@ -17289,7 +17311,7 @@
         <v>2.0171123328217101E-4</v>
       </c>
     </row>
-    <row r="119" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A119" s="26" t="s">
         <v>61</v>
       </c>
@@ -17341,7 +17363,7 @@
         <v>9.0585048121064743E-4</v>
       </c>
     </row>
-    <row r="120" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A120" s="26" t="s">
         <v>61</v>
       </c>
@@ -17395,7 +17417,7 @@
         <v>5.5895604583549826E-4</v>
       </c>
     </row>
-    <row r="121" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A121" s="26" t="s">
         <v>61</v>
       </c>
@@ -17449,7 +17471,7 @@
         <v>5.9586647863810009E-4</v>
       </c>
     </row>
-    <row r="122" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A122" s="30" t="s">
         <v>61</v>
       </c>
@@ -17503,7 +17525,7 @@
         <v>5.9395027360884304E-4</v>
       </c>
     </row>
-    <row r="123" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A123" s="26" t="s">
         <v>61</v>
       </c>
@@ -17557,7 +17579,7 @@
         <v>5.6497696684834598E-4</v>
       </c>
     </row>
-    <row r="124" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A124" s="30" t="s">
         <v>61</v>
       </c>
@@ -17611,7 +17633,7 @@
         <v>5.1862725905372977E-4</v>
       </c>
     </row>
-    <row r="125" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A125" s="26" t="s">
         <v>61</v>
       </c>
@@ -17665,7 +17687,7 @@
         <v>3.2173814470789232E-5</v>
       </c>
     </row>
-    <row r="126" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A126" s="30" t="s">
         <v>61</v>
       </c>
@@ -17719,7 +17741,7 @@
         <v>3.2173814470789232E-5</v>
       </c>
     </row>
-    <row r="127" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A127" s="30" t="s">
         <v>61</v>
       </c>
@@ -17773,7 +17795,7 @@
         <v>3.4334205407993363E-5</v>
       </c>
     </row>
-    <row r="128" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A128" s="30" t="s">
         <v>61</v>
       </c>
@@ -17827,7 +17849,7 @@
         <v>2.1042825374402833E-5</v>
       </c>
     </row>
-    <row r="129" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A129" s="26" t="s">
         <v>61</v>
       </c>
@@ -17881,7 +17903,7 @@
         <v>7.5811156020801356E-8</v>
       </c>
     </row>
-    <row r="130" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A130" s="26" t="s">
         <v>61</v>
       </c>
@@ -17935,7 +17957,7 @@
         <v>4.2003281817037876E-4</v>
       </c>
     </row>
-    <row r="131" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A131" s="26" t="s">
         <v>61</v>
       </c>
@@ -17989,7 +18011,7 @@
         <v>4.5897773477486449E-4</v>
       </c>
     </row>
-    <row r="132" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A132" s="26" t="s">
         <v>61</v>
       </c>
@@ -18033,7 +18055,7 @@
         <v>9.8407805442712548E-5</v>
       </c>
     </row>
-    <row r="133" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A133" s="26" t="s">
         <v>61</v>
       </c>
@@ -18077,7 +18099,7 @@
         <v>9.6537344525351703E-5</v>
       </c>
     </row>
-    <row r="134" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A134" s="30" t="s">
         <v>61</v>
       </c>
@@ -18131,7 +18153,7 @@
         <v>9.2359833137233124E-4</v>
       </c>
     </row>
-    <row r="135" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A135" s="30" t="s">
         <v>61</v>
       </c>
@@ -18185,14 +18207,9 @@
         <v>1.2124619343610176E-3</v>
       </c>
     </row>
-    <row r="136" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="136" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <autoFilter ref="A2:P136" xr:uid="{00000000-0001-0000-0400-000000000000}">
-    <filterColumn colId="3">
-      <filters>
-        <filter val="2024"/>
-      </filters>
-    </filterColumn>
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:P136">
       <sortCondition ref="B2:B136"/>
     </sortState>
@@ -18223,24 +18240,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="91" t="s">
+      <c r="A1" s="92" t="s">
         <v>56</v>
       </c>
-      <c r="B1" s="76"/>
-      <c r="C1" s="76"/>
-      <c r="D1" s="76"/>
-      <c r="E1" s="76"/>
-      <c r="F1" s="76"/>
-      <c r="G1" s="76"/>
-      <c r="H1" s="76"/>
-      <c r="I1" s="76"/>
-      <c r="J1" s="76"/>
-      <c r="K1" s="76"/>
-      <c r="L1" s="76"/>
-      <c r="M1" s="76"/>
-      <c r="N1" s="76"/>
-      <c r="O1" s="76"/>
-      <c r="P1" s="76"/>
+      <c r="B1" s="77"/>
+      <c r="C1" s="77"/>
+      <c r="D1" s="77"/>
+      <c r="E1" s="77"/>
+      <c r="F1" s="77"/>
+      <c r="G1" s="77"/>
+      <c r="H1" s="77"/>
+      <c r="I1" s="77"/>
+      <c r="J1" s="77"/>
+      <c r="K1" s="77"/>
+      <c r="L1" s="77"/>
+      <c r="M1" s="77"/>
+      <c r="N1" s="77"/>
+      <c r="O1" s="77"/>
+      <c r="P1" s="77"/>
     </row>
     <row r="2" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="32" t="s">
@@ -23331,16 +23348,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="96" t="s">
+      <c r="A1" s="97" t="s">
         <v>144</v>
       </c>
-      <c r="B1" s="76"/>
-      <c r="C1" s="76"/>
-      <c r="D1" s="76"/>
-      <c r="E1" s="76"/>
-      <c r="F1" s="76"/>
-      <c r="G1" s="76"/>
-      <c r="H1" s="76"/>
+      <c r="B1" s="77"/>
+      <c r="C1" s="77"/>
+      <c r="D1" s="77"/>
+      <c r="E1" s="77"/>
+      <c r="F1" s="77"/>
+      <c r="G1" s="77"/>
+      <c r="H1" s="77"/>
     </row>
     <row r="2" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="33" t="s">
@@ -44122,23 +44139,23 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:17" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A1" s="80" t="s">
+      <c r="A1" s="76" t="s">
         <v>2022</v>
       </c>
-      <c r="B1" s="76"/>
-      <c r="C1" s="76"/>
-      <c r="D1" s="76"/>
-      <c r="E1" s="76"/>
-      <c r="F1" s="76"/>
-      <c r="G1" s="76"/>
-      <c r="H1" s="76"/>
-      <c r="I1" s="76"/>
-      <c r="J1" s="76"/>
-      <c r="K1" s="76"/>
-      <c r="L1" s="76"/>
-      <c r="M1" s="76"/>
-      <c r="N1" s="76"/>
-      <c r="O1" s="76"/>
+      <c r="B1" s="77"/>
+      <c r="C1" s="77"/>
+      <c r="D1" s="77"/>
+      <c r="E1" s="77"/>
+      <c r="F1" s="77"/>
+      <c r="G1" s="77"/>
+      <c r="H1" s="77"/>
+      <c r="I1" s="77"/>
+      <c r="J1" s="77"/>
+      <c r="K1" s="77"/>
+      <c r="L1" s="77"/>
+      <c r="M1" s="77"/>
+      <c r="N1" s="77"/>
+      <c r="O1" s="77"/>
     </row>
     <row r="2" spans="1:17" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A2" s="63" t="s">
@@ -44879,41 +44896,41 @@
       </c>
     </row>
     <row r="15" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="B15" s="100"/>
-      <c r="E15" s="97" t="s">
+      <c r="B15" s="75"/>
+      <c r="E15" s="98" t="s">
         <v>2034</v>
       </c>
-      <c r="F15" s="97"/>
-      <c r="G15" s="97"/>
-      <c r="H15" s="97"/>
-      <c r="I15" s="97"/>
-      <c r="J15" s="97"/>
-      <c r="K15" s="97"/>
-      <c r="L15" s="97"/>
-      <c r="M15" s="97"/>
-      <c r="N15" s="97"/>
-      <c r="O15" s="97"/>
-      <c r="P15" s="97"/>
-      <c r="Q15" s="97"/>
+      <c r="F15" s="98"/>
+      <c r="G15" s="98"/>
+      <c r="H15" s="98"/>
+      <c r="I15" s="98"/>
+      <c r="J15" s="98"/>
+      <c r="K15" s="98"/>
+      <c r="L15" s="98"/>
+      <c r="M15" s="98"/>
+      <c r="N15" s="98"/>
+      <c r="O15" s="98"/>
+      <c r="P15" s="98"/>
+      <c r="Q15" s="98"/>
     </row>
     <row r="16" spans="1:17" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A16" s="98" t="s">
+      <c r="A16" s="99" t="s">
         <v>2032</v>
       </c>
-      <c r="B16" s="98"/>
-      <c r="C16" s="98"/>
-      <c r="D16" s="98"/>
-      <c r="E16" s="98"/>
-      <c r="F16" s="98"/>
-      <c r="G16" s="98"/>
-      <c r="H16" s="98"/>
-      <c r="I16" s="98"/>
-      <c r="J16" s="98"/>
-      <c r="K16" s="98"/>
-      <c r="L16" s="98"/>
-      <c r="M16" s="98"/>
-      <c r="N16" s="98"/>
-      <c r="O16" s="98"/>
+      <c r="B16" s="99"/>
+      <c r="C16" s="99"/>
+      <c r="D16" s="99"/>
+      <c r="E16" s="99"/>
+      <c r="F16" s="99"/>
+      <c r="G16" s="99"/>
+      <c r="H16" s="99"/>
+      <c r="I16" s="99"/>
+      <c r="J16" s="99"/>
+      <c r="K16" s="99"/>
+      <c r="L16" s="99"/>
+      <c r="M16" s="99"/>
+      <c r="N16" s="99"/>
+      <c r="O16" s="99"/>
     </row>
     <row r="17" spans="1:15" ht="24" x14ac:dyDescent="0.3">
       <c r="A17" s="66" t="s">
@@ -45622,17 +45639,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="99" t="s">
+      <c r="A1" s="100" t="s">
         <v>2041</v>
       </c>
-      <c r="B1" s="99"/>
-      <c r="C1" s="99"/>
-      <c r="D1" s="99"/>
-      <c r="E1" s="99"/>
-      <c r="F1" s="99"/>
-      <c r="G1" s="99"/>
-      <c r="H1" s="99"/>
-      <c r="I1" s="99"/>
+      <c r="B1" s="100"/>
+      <c r="C1" s="100"/>
+      <c r="D1" s="100"/>
+      <c r="E1" s="100"/>
+      <c r="F1" s="100"/>
+      <c r="G1" s="100"/>
+      <c r="H1" s="100"/>
+      <c r="I1" s="100"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" s="74" t="s">

</xml_diff>